<commit_message>
Resync 28 published packets against a corpus-wide mtime staleness bug
A prior enrichment pass edited case.md across most published cases but
never rebuilt their docx/xlsx/html packets, so a live Tier 1 re-check
flagged 28 cases (of 39 that should be clean) as CONTINUITY STALE. Verified
each individually (content-hash match against MANIFEST, direct docx/xlsx/html
diff against current case.md, and a rendered-PDF read for facilitator-content
leaks) before touching anything: 27 were pure mtime noise with no real content
drift, and apron-order had one small real edit that needed an actual rebuild.
All 39 now pass a live Tier 1 re-check with 0 blockers.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cases/apron-order/published/Apron Order - Data.xlsx
+++ b/cases/apron-order/published/Apron Order - Data.xlsx
@@ -32,28 +32,23 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDDDDD"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -68,11 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -442,8 +436,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,7 +446,6 @@
           <t>Apron Order -- Data Workbook</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -540,13 +533,12 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="n"/>
       <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Value</t>
@@ -597,7 +589,6 @@
       <c r="B4" s="2" t="n">
         <v>22.5</v>
       </c>
-      <c r="C4" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -619,7 +610,6 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="n"/>
       <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Value</t>
@@ -662,9 +652,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -678,7 +668,6 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="C1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -691,7 +680,6 @@
           <t>24 3/8</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -704,7 +692,6 @@
           <t>28 1/2</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -717,7 +704,6 @@
           <t>2/3 x body panel width -- see Challenge D1</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -730,7 +716,6 @@
           <t>36 5/8</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -743,15 +728,8 @@
           <t>1 3/8</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Cut on the Fold</t>
@@ -824,13 +802,12 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="n"/>
       <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Value</t>
@@ -866,7 +843,6 @@
       <c r="B3" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="C3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -882,11 +858,11 @@
   <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>D1 -- Waist Tie Length</t>
         </is>
@@ -899,11 +875,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-    </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>D2 -- Trimmed Marker Length</t>
         </is>
@@ -916,11 +889,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-    </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>D3 -- Aprons Per Bolt</t>
         </is>
@@ -933,11 +903,8 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>D4 -- Splitting a Remnant</t>
         </is>
@@ -950,11 +917,8 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>D5 -- Comparing Waste</t>
         </is>
@@ -967,11 +931,8 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>D6 -- The Hem Check</t>
         </is>
@@ -984,11 +945,8 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>D7 -- A Total Cost Verdict</t>
         </is>
@@ -1037,7 +995,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Dollar difference</t>
         </is>

</xml_diff>